<commit_message>
update for html file
</commit_message>
<xml_diff>
--- a/src/test/resources/RegisterData/Register_TestData.xlsx
+++ b/src/test/resources/RegisterData/Register_TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30516"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9C474534-511F-4D21-A86A-4DD723862247}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{58C51DEE-910C-40ED-BFB6-2360748EF18A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="550" uniqueCount="239">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -42,22 +42,22 @@
     <t>Scenario</t>
   </si>
   <si>
-    <t>First Name</t>
-  </si>
-  <si>
-    <t>Last Name</t>
+    <t>FirstName</t>
+  </si>
+  <si>
+    <t>LastName</t>
   </si>
   <si>
     <t>Email</t>
   </si>
   <si>
-    <t>Phone Number</t>
+    <t>Phone</t>
   </si>
   <si>
     <t>Password</t>
   </si>
   <si>
-    <t>Repeat Password</t>
+    <t>RepeatPassword</t>
   </si>
   <si>
     <t>Terms</t>
@@ -69,616 +69,658 @@
     <t>REG-001</t>
   </si>
   <si>
-    <t>Valid registration</t>
+    <t>Valid registration - new user</t>
+  </si>
+  <si>
+    <t>Rahul</t>
+  </si>
+  <si>
+    <t>Nair</t>
+  </si>
+  <si>
+    <t>rahul.reg061@shopease.com</t>
+  </si>
+  <si>
+    <t>Rahul@123</t>
+  </si>
+  <si>
+    <t>Checked</t>
+  </si>
+  <si>
+    <t>SUCCESS</t>
+  </si>
+  <si>
+    <t>REG-002</t>
+  </si>
+  <si>
+    <t>Valid registration - different name</t>
+  </si>
+  <si>
+    <t>Meera</t>
+  </si>
+  <si>
+    <t>Menon</t>
+  </si>
+  <si>
+    <t>meera.reg062@shopease.com</t>
+  </si>
+  <si>
+    <t>Meera@123</t>
+  </si>
+  <si>
+    <t>REG-003</t>
+  </si>
+  <si>
+    <t>Valid registration - mixed case name</t>
+  </si>
+  <si>
+    <t>aRJuN</t>
+  </si>
+  <si>
+    <t>Kumar</t>
+  </si>
+  <si>
+    <t>arjun.reg063@shopease.com</t>
+  </si>
+  <si>
+    <t>Arjun@123</t>
+  </si>
+  <si>
+    <t>REG-004</t>
+  </si>
+  <si>
+    <t>First name minimum boundary</t>
+  </si>
+  <si>
+    <t>Ab</t>
+  </si>
+  <si>
+    <t>Thomas</t>
+  </si>
+  <si>
+    <t>ab.reg064@shopease.com</t>
+  </si>
+  <si>
+    <t>Test@123</t>
+  </si>
+  <si>
+    <t>EDGE</t>
+  </si>
+  <si>
+    <t>REG-005</t>
+  </si>
+  <si>
+    <t>Last name minimum boundary</t>
+  </si>
+  <si>
+    <t>Arun</t>
+  </si>
+  <si>
+    <t>Li</t>
+  </si>
+  <si>
+    <t>arun.reg065@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-006</t>
+  </si>
+  <si>
+    <t>First name maximum length</t>
+  </si>
+  <si>
+    <t>AAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
+  </si>
+  <si>
+    <t>longfirst.reg066@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-007</t>
+  </si>
+  <si>
+    <t>Last name maximum length</t>
+  </si>
+  <si>
+    <t>BBBBBBBBBBBBBBBBBBBBBBBBBBBBBB</t>
+  </si>
+  <si>
+    <t>longlast.reg067@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-008</t>
+  </si>
+  <si>
+    <t>First name with numeric suffix</t>
+  </si>
+  <si>
+    <t>Arun2</t>
+  </si>
+  <si>
+    <t>arun.reg068@shopease.com</t>
+  </si>
+  <si>
+    <t>VALIDATION</t>
+  </si>
+  <si>
+    <t>REG-009</t>
+  </si>
+  <si>
+    <t>First name with multiple spaces</t>
+  </si>
+  <si>
+    <t>Arun Kumar</t>
+  </si>
+  <si>
+    <t>arun.reg069@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-010</t>
+  </si>
+  <si>
+    <t>Last name with multiple spaces</t>
+  </si>
+  <si>
+    <t>Nair Kumar</t>
+  </si>
+  <si>
+    <t>arun.reg070@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-011</t>
+  </si>
+  <si>
+    <t>Email with subdomain</t>
+  </si>
+  <si>
+    <t>arun.reg071@mail.shopease.com</t>
+  </si>
+  <si>
+    <t>REG-012</t>
+  </si>
+  <si>
+    <t>Email with plus alias</t>
+  </si>
+  <si>
+    <t>arun+test072@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-013</t>
+  </si>
+  <si>
+    <t>Email with underscore</t>
+  </si>
+  <si>
+    <t>arun_test073@shopease.com</t>
+  </si>
+  <si>
+    <t>SUCCESS/EDGE</t>
+  </si>
+  <si>
+    <t>REG-014</t>
+  </si>
+  <si>
+    <t>Email with hyphen</t>
+  </si>
+  <si>
+    <t>arun-test074@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-015</t>
+  </si>
+  <si>
+    <t>Email with multiple dots</t>
+  </si>
+  <si>
+    <t>arun.test.075@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-016</t>
+  </si>
+  <si>
+    <t>Email with double @</t>
+  </si>
+  <si>
+    <t>arun@@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-017</t>
+  </si>
+  <si>
+    <t>Email with dot before @</t>
+  </si>
+  <si>
+    <t>arun.076.@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-018</t>
+  </si>
+  <si>
+    <t>Email starting with @</t>
+  </si>
+  <si>
+    <t>@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-019</t>
+  </si>
+  <si>
+    <t>Email ending with @</t>
+  </si>
+  <si>
+    <t>arun079@</t>
+  </si>
+  <si>
+    <t>REG-020</t>
+  </si>
+  <si>
+    <t>Password exactly 6 characters</t>
+  </si>
+  <si>
+    <t>arun.reg080@shopease.com</t>
+  </si>
+  <si>
+    <t>Abc@12</t>
+  </si>
+  <si>
+    <t>REG-021</t>
+  </si>
+  <si>
+    <t>Password 5 characters</t>
+  </si>
+  <si>
+    <t>arun.reg081@shopease.com</t>
+  </si>
+  <si>
+    <t>Abc@1</t>
+  </si>
+  <si>
+    <t>REG-022</t>
+  </si>
+  <si>
+    <t>Password with uppercase lowercase number special</t>
+  </si>
+  <si>
+    <t>arun.reg082@shopease.com</t>
+  </si>
+  <si>
+    <t>ArUn@123</t>
+  </si>
+  <si>
+    <t>REG-023</t>
+  </si>
+  <si>
+    <t>Password leading space</t>
+  </si>
+  <si>
+    <t>arun.reg083@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-024</t>
+  </si>
+  <si>
+    <t>Password trailing space</t>
+  </si>
+  <si>
+    <t>arun.reg084@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-025</t>
+  </si>
+  <si>
+    <t>Repeat password leading space</t>
+  </si>
+  <si>
+    <t>arun.reg085@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-026</t>
+  </si>
+  <si>
+    <t>Repeat password trailing space</t>
+  </si>
+  <si>
+    <t>arun.reg086@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-027</t>
+  </si>
+  <si>
+    <t>Phone starts with zero</t>
+  </si>
+  <si>
+    <t>arun.reg087@shopease.com</t>
+  </si>
+  <si>
+    <t>EDGE/VALIDATION</t>
+  </si>
+  <si>
+    <t>REG-028</t>
+  </si>
+  <si>
+    <t>Phone with spaces</t>
+  </si>
+  <si>
+    <t>arun.reg088@shopease.com</t>
+  </si>
+  <si>
+    <t>98765 43210</t>
+  </si>
+  <si>
+    <t>REG-029</t>
+  </si>
+  <si>
+    <t>Phone with leading plus</t>
+  </si>
+  <si>
+    <t>arun.reg089@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-030</t>
+  </si>
+  <si>
+    <t>Valid registration after invalid data correction</t>
+  </si>
+  <si>
+    <t>Priya</t>
+  </si>
+  <si>
+    <t>Raj</t>
+  </si>
+  <si>
+    <t>priya.reg090@shopease.com</t>
+  </si>
+  <si>
+    <t>Priya@123</t>
+  </si>
+  <si>
+    <t>REG-031</t>
+  </si>
+  <si>
+    <t>Terms checkbox checked</t>
   </si>
   <si>
     <t>Aswin</t>
   </si>
   <si>
-    <t>Kumar</t>
-  </si>
-  <si>
-    <t>aswin.reg001@shopease.com</t>
-  </si>
-  <si>
-    <t>Test@123</t>
-  </si>
-  <si>
-    <t>Checked</t>
-  </si>
-  <si>
-    <t>SUCCESS</t>
-  </si>
-  <si>
-    <t>REG-002</t>
-  </si>
-  <si>
-    <t>Valid registration with optional phone blank</t>
-  </si>
-  <si>
-    <t>aswin.reg002@shopease.com</t>
-  </si>
-  <si>
-    <t>REG-003</t>
-  </si>
-  <si>
-    <t>Empty first name</t>
-  </si>
-  <si>
-    <t>aswin.reg003@shopease.com</t>
-  </si>
-  <si>
-    <t>VALIDATION</t>
-  </si>
-  <si>
-    <t>REG-004</t>
-  </si>
-  <si>
-    <t>Empty last name</t>
-  </si>
-  <si>
-    <t>aswin.reg004@shopease.com</t>
-  </si>
-  <si>
-    <t>REG-005</t>
-  </si>
-  <si>
-    <t>Empty email</t>
-  </si>
-  <si>
-    <t>REG-006</t>
-  </si>
-  <si>
-    <t>Empty password</t>
-  </si>
-  <si>
-    <t>aswin.reg006@shopease.com</t>
-  </si>
-  <si>
-    <t>REG-007</t>
-  </si>
-  <si>
-    <t>Empty repeat password</t>
-  </si>
-  <si>
-    <t>aswin.reg007@shopease.com</t>
-  </si>
-  <si>
-    <t>REG-008</t>
-  </si>
-  <si>
-    <t>All mandatory fields empty</t>
-  </si>
-  <si>
-    <t>Unchecked</t>
-  </si>
-  <si>
-    <t>REG-009</t>
-  </si>
-  <si>
-    <t>Invalid email format</t>
-  </si>
-  <si>
-    <t>aswin.reg009</t>
-  </si>
-  <si>
-    <t>REG-010</t>
-  </si>
-  <si>
-    <t>Email without domain</t>
-  </si>
-  <si>
-    <t>aswin@</t>
-  </si>
-  <si>
-    <t>REG-011</t>
-  </si>
-  <si>
-    <t>Email without @</t>
-  </si>
-  <si>
-    <t>aswin.gmail.com</t>
-  </si>
-  <si>
-    <t>REG-012</t>
-  </si>
-  <si>
-    <t>Email with spaces</t>
-  </si>
-  <si>
-    <t>aswin test@gmail.com</t>
-  </si>
-  <si>
-    <t>REG-013</t>
-  </si>
-  <si>
-    <t>Valid email with uppercase characters</t>
-  </si>
-  <si>
-    <t>ASWIN.REG013@SHOPEASE.COM</t>
-  </si>
-  <si>
-    <t>SUCCESS/VALIDATION</t>
-  </si>
-  <si>
-    <t>REG-014</t>
-  </si>
-  <si>
-    <t>Email with leading space</t>
-  </si>
-  <si>
-    <t>aswin.reg014@shopease.com</t>
-  </si>
-  <si>
-    <t>EDGE</t>
-  </si>
-  <si>
-    <t>REG-015</t>
-  </si>
-  <si>
-    <t>Email with trailing space</t>
-  </si>
-  <si>
-    <t>aswin.reg015@shopease.com</t>
-  </si>
-  <si>
-    <t>REG-016</t>
-  </si>
-  <si>
-    <t>Duplicate account creation</t>
-  </si>
-  <si>
-    <t>existing.user@shopease.com</t>
-  </si>
-  <si>
-    <t>FAILURE</t>
-  </si>
-  <si>
-    <t>REG-017</t>
-  </si>
-  <si>
-    <t>Duplicate email with different name</t>
-  </si>
-  <si>
-    <t>Rahul</t>
-  </si>
-  <si>
-    <t>Sharma</t>
-  </si>
-  <si>
-    <t>Rahul@123</t>
-  </si>
-  <si>
-    <t>REG-018</t>
-  </si>
-  <si>
-    <t>Duplicate email with different password</t>
-  </si>
-  <si>
-    <t>New@123</t>
-  </si>
-  <si>
-    <t>REG-019</t>
-  </si>
-  <si>
-    <t>Password and repeat password match</t>
-  </si>
-  <si>
-    <t>aswin.reg019@shopease.com</t>
-  </si>
-  <si>
-    <t>REG-020</t>
-  </si>
-  <si>
-    <t>Password and repeat password mismatch</t>
-  </si>
-  <si>
-    <t>aswin.reg020@shopease.com</t>
+    <t>aswin.reg031@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-032</t>
+  </si>
+  <si>
+    <t>First name with numbers</t>
+  </si>
+  <si>
+    <t>Aswin123</t>
+  </si>
+  <si>
+    <t>aswin.reg032@shopease.com</t>
+  </si>
+  <si>
+    <t>VALIDATION/EDGE</t>
+  </si>
+  <si>
+    <t>REG-033</t>
+  </si>
+  <si>
+    <t>First name with special characters</t>
+  </si>
+  <si>
+    <t>Aswin@</t>
+  </si>
+  <si>
+    <t>aswin.reg033@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-034</t>
+  </si>
+  <si>
+    <t>Last name with numbers</t>
+  </si>
+  <si>
+    <t>Kumar123</t>
+  </si>
+  <si>
+    <t>aswin.reg034@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-035</t>
+  </si>
+  <si>
+    <t>Name with hyphen</t>
+  </si>
+  <si>
+    <t>Anne-Marie</t>
+  </si>
+  <si>
+    <t>anne.reg035@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-036</t>
+  </si>
+  <si>
+    <t>Name with apostrophe</t>
+  </si>
+  <si>
+    <t>O'Brien</t>
+  </si>
+  <si>
+    <t>obrien.reg036@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-037</t>
+  </si>
+  <si>
+    <t>Single-character first name</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>aswin.reg037@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-038</t>
+  </si>
+  <si>
+    <t>Single-character last name</t>
+  </si>
+  <si>
+    <t>K</t>
+  </si>
+  <si>
+    <t>aswin.reg038@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-039</t>
+  </si>
+  <si>
+    <t>Phone number valid</t>
+  </si>
+  <si>
+    <t>aswin.reg039@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-040</t>
+  </si>
+  <si>
+    <t>Phone number less than expected length</t>
+  </si>
+  <si>
+    <t>aswin.reg040@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-041</t>
+  </si>
+  <si>
+    <t>Phone number more than expected length</t>
+  </si>
+  <si>
+    <t>aswin.reg041@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-042</t>
+  </si>
+  <si>
+    <t>Phone contains alphabets</t>
+  </si>
+  <si>
+    <t>aswin.reg042@shopease.com</t>
+  </si>
+  <si>
+    <t>98765abc10</t>
+  </si>
+  <si>
+    <t>REG-043</t>
+  </si>
+  <si>
+    <t>Phone contains special characters</t>
+  </si>
+  <si>
+    <t>aswin.reg043@shopease.com</t>
+  </si>
+  <si>
+    <t>98765@3210</t>
+  </si>
+  <si>
+    <t>REG-044</t>
+  </si>
+  <si>
+    <t>Phone with country code</t>
+  </si>
+  <si>
+    <t>aswin.reg044@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-045</t>
+  </si>
+  <si>
+    <t>Phone all zeros</t>
+  </si>
+  <si>
+    <t>aswin.reg045@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-046</t>
+  </si>
+  <si>
+    <t>First name with leading space</t>
+  </si>
+  <si>
+    <t>aswin.reg046@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-047</t>
+  </si>
+  <si>
+    <t>Last name with trailing space</t>
+  </si>
+  <si>
+    <t>aswin.reg047@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-048</t>
+  </si>
+  <si>
+    <t>Double-click Create Account</t>
+  </si>
+  <si>
+    <t>aswin.reg048@shopease.com</t>
+  </si>
+  <si>
+    <t>ONE ACCOUNT ONLY</t>
+  </si>
+  <si>
+    <t>REG-049</t>
+  </si>
+  <si>
+    <t>Submit same registration repeatedly</t>
+  </si>
+  <si>
+    <t>aswin.reg049@shopease.com</t>
+  </si>
+  <si>
+    <t>DUPLICATE BLOCKED</t>
+  </si>
+  <si>
+    <t>REG-050</t>
+  </si>
+  <si>
+    <t>SQL injection in first name</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> OR 1=1 --</t>
+  </si>
+  <si>
+    <t>aswin.reg050@shopease.com</t>
+  </si>
+  <si>
+    <t>VALIDATION/SAFE</t>
+  </si>
+  <si>
+    <t>REG-051</t>
+  </si>
+  <si>
+    <t>Script injection in first name</t>
+  </si>
+  <si>
+    <t>&lt;script&gt;alert(1)&lt;/script&gt;</t>
+  </si>
+  <si>
+    <t>aswin.reg051@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-052</t>
+  </si>
+  <si>
+    <t>Script injection in email</t>
+  </si>
+  <si>
+    <t>REG-053</t>
+  </si>
+  <si>
+    <t>Spaces only in first name</t>
+  </si>
+  <si>
+    <t>aswin.reg053@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-054</t>
+  </si>
+  <si>
+    <t>Spaces only in last name</t>
+  </si>
+  <si>
+    <t>aswin.reg054@shopease.com</t>
+  </si>
+  <si>
+    <t>REG-055</t>
+  </si>
+  <si>
+    <t>Spaces only in email</t>
+  </si>
+  <si>
+    <t>REG-056</t>
+  </si>
+  <si>
+    <t>Browser refresh after entering data</t>
+  </si>
+  <si>
+    <t>aswin.reg056@shopease.com</t>
+  </si>
+  <si>
+    <t>STATE HANDLING</t>
+  </si>
+  <si>
+    <t>REG-057</t>
+  </si>
+  <si>
+    <t>Registration after failed attempt</t>
+  </si>
+  <si>
+    <t>aswin.reg057@shopease.com</t>
   </si>
   <si>
     <t>Test@124</t>
-  </si>
-  <si>
-    <t>REG-021</t>
-  </si>
-  <si>
-    <t>Repeat password differs by case</t>
-  </si>
-  <si>
-    <t>aswin.reg021@shopease.com</t>
-  </si>
-  <si>
-    <t>test@123</t>
-  </si>
-  <si>
-    <t>REG-022</t>
-  </si>
-  <si>
-    <t>Repeat password completely different</t>
-  </si>
-  <si>
-    <t>aswin.reg022@shopease.com</t>
-  </si>
-  <si>
-    <t>Wrong@123</t>
-  </si>
-  <si>
-    <t>REG-023</t>
-  </si>
-  <si>
-    <t>Password minimum length</t>
-  </si>
-  <si>
-    <t>aswin.reg023@shopease.com</t>
-  </si>
-  <si>
-    <t>Test@1</t>
-  </si>
-  <si>
-    <t>REG-024</t>
-  </si>
-  <si>
-    <t>Password below minimum length</t>
-  </si>
-  <si>
-    <t>aswin.reg024@shopease.com</t>
-  </si>
-  <si>
-    <t>Test1</t>
-  </si>
-  <si>
-    <t>REG-025</t>
-  </si>
-  <si>
-    <t>Password numeric only</t>
-  </si>
-  <si>
-    <t>aswin.reg025@shopease.com</t>
-  </si>
-  <si>
-    <t>REG-026</t>
-  </si>
-  <si>
-    <t>Password alphabetic only</t>
-  </si>
-  <si>
-    <t>aswin.reg026@shopease.com</t>
-  </si>
-  <si>
-    <t>abcdef</t>
-  </si>
-  <si>
-    <t>REG-027</t>
-  </si>
-  <si>
-    <t>Password special characters</t>
-  </si>
-  <si>
-    <t>aswin.reg027@shopease.com</t>
-  </si>
-  <si>
-    <t>@#$%^&amp;</t>
-  </si>
-  <si>
-    <t>REG-028</t>
-  </si>
-  <si>
-    <t>Password with spaces</t>
-  </si>
-  <si>
-    <t>aswin.reg028@shopease.com</t>
-  </si>
-  <si>
-    <t>Test @123</t>
-  </si>
-  <si>
-    <t>REG-029</t>
-  </si>
-  <si>
-    <t>Very long password</t>
-  </si>
-  <si>
-    <t>aswin.reg029@shopease.com</t>
-  </si>
-  <si>
-    <t>AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
-  </si>
-  <si>
-    <t>REG-030</t>
-  </si>
-  <si>
-    <t>Terms checkbox unchecked</t>
-  </si>
-  <si>
-    <t>aswin.reg030@shopease.com</t>
-  </si>
-  <si>
-    <t>REG-031</t>
-  </si>
-  <si>
-    <t>Terms checkbox checked</t>
-  </si>
-  <si>
-    <t>aswin.reg031@shopease.com</t>
-  </si>
-  <si>
-    <t>REG-032</t>
-  </si>
-  <si>
-    <t>First name with numbers</t>
-  </si>
-  <si>
-    <t>Aswin123</t>
-  </si>
-  <si>
-    <t>aswin.reg032@shopease.com</t>
-  </si>
-  <si>
-    <t>VALIDATION/EDGE</t>
-  </si>
-  <si>
-    <t>REG-033</t>
-  </si>
-  <si>
-    <t>First name with special characters</t>
-  </si>
-  <si>
-    <t>Aswin@</t>
-  </si>
-  <si>
-    <t>aswin.reg033@shopease.com</t>
-  </si>
-  <si>
-    <t>REG-034</t>
-  </si>
-  <si>
-    <t>Last name with numbers</t>
-  </si>
-  <si>
-    <t>Kumar123</t>
-  </si>
-  <si>
-    <t>aswin.reg034@shopease.com</t>
-  </si>
-  <si>
-    <t>REG-035</t>
-  </si>
-  <si>
-    <t>Name with hyphen</t>
-  </si>
-  <si>
-    <t>Anne-Marie</t>
-  </si>
-  <si>
-    <t>Thomas</t>
-  </si>
-  <si>
-    <t>anne.reg035@shopease.com</t>
-  </si>
-  <si>
-    <t>REG-036</t>
-  </si>
-  <si>
-    <t>Name with apostrophe</t>
-  </si>
-  <si>
-    <t>O'Brien</t>
-  </si>
-  <si>
-    <t>obrien.reg036@shopease.com</t>
-  </si>
-  <si>
-    <t>REG-037</t>
-  </si>
-  <si>
-    <t>Single-character first name</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>aswin.reg037@shopease.com</t>
-  </si>
-  <si>
-    <t>REG-038</t>
-  </si>
-  <si>
-    <t>Single-character last name</t>
-  </si>
-  <si>
-    <t>K</t>
-  </si>
-  <si>
-    <t>aswin.reg038@shopease.com</t>
-  </si>
-  <si>
-    <t>REG-039</t>
-  </si>
-  <si>
-    <t>Phone number valid</t>
-  </si>
-  <si>
-    <t>aswin.reg039@shopease.com</t>
-  </si>
-  <si>
-    <t>REG-040</t>
-  </si>
-  <si>
-    <t>Phone number less than expected length</t>
-  </si>
-  <si>
-    <t>aswin.reg040@shopease.com</t>
-  </si>
-  <si>
-    <t>REG-041</t>
-  </si>
-  <si>
-    <t>Phone number more than expected length</t>
-  </si>
-  <si>
-    <t>aswin.reg041@shopease.com</t>
-  </si>
-  <si>
-    <t>REG-042</t>
-  </si>
-  <si>
-    <t>Phone contains alphabets</t>
-  </si>
-  <si>
-    <t>aswin.reg042@shopease.com</t>
-  </si>
-  <si>
-    <t>98765abc10</t>
-  </si>
-  <si>
-    <t>REG-043</t>
-  </si>
-  <si>
-    <t>Phone contains special characters</t>
-  </si>
-  <si>
-    <t>aswin.reg043@shopease.com</t>
-  </si>
-  <si>
-    <t>98765@3210</t>
-  </si>
-  <si>
-    <t>REG-044</t>
-  </si>
-  <si>
-    <t>Phone with country code</t>
-  </si>
-  <si>
-    <t>aswin.reg044@shopease.com</t>
-  </si>
-  <si>
-    <t>REG-045</t>
-  </si>
-  <si>
-    <t>Phone all zeros</t>
-  </si>
-  <si>
-    <t>aswin.reg045@shopease.com</t>
-  </si>
-  <si>
-    <t>REG-046</t>
-  </si>
-  <si>
-    <t>First name with leading space</t>
-  </si>
-  <si>
-    <t>aswin.reg046@shopease.com</t>
-  </si>
-  <si>
-    <t>REG-047</t>
-  </si>
-  <si>
-    <t>Last name with trailing space</t>
-  </si>
-  <si>
-    <t>aswin.reg047@shopease.com</t>
-  </si>
-  <si>
-    <t>REG-048</t>
-  </si>
-  <si>
-    <t>Double-click Create Account</t>
-  </si>
-  <si>
-    <t>aswin.reg048@shopease.com</t>
-  </si>
-  <si>
-    <t>ONE ACCOUNT ONLY</t>
-  </si>
-  <si>
-    <t>REG-049</t>
-  </si>
-  <si>
-    <t>Submit same registration repeatedly</t>
-  </si>
-  <si>
-    <t>aswin.reg049@shopease.com</t>
-  </si>
-  <si>
-    <t>DUPLICATE BLOCKED</t>
-  </si>
-  <si>
-    <t>REG-050</t>
-  </si>
-  <si>
-    <t>SQL injection in first name</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> OR 1=1 --</t>
-  </si>
-  <si>
-    <t>aswin.reg050@shopease.com</t>
-  </si>
-  <si>
-    <t>VALIDATION/SAFE</t>
-  </si>
-  <si>
-    <t>REG-051</t>
-  </si>
-  <si>
-    <t>Script injection in first name</t>
-  </si>
-  <si>
-    <t>&lt;script&gt;alert(1)&lt;/script&gt;</t>
-  </si>
-  <si>
-    <t>aswin.reg051@shopease.com</t>
-  </si>
-  <si>
-    <t>REG-052</t>
-  </si>
-  <si>
-    <t>Script injection in email</t>
-  </si>
-  <si>
-    <t>REG-053</t>
-  </si>
-  <si>
-    <t>Spaces only in first name</t>
-  </si>
-  <si>
-    <t>aswin.reg053@shopease.com</t>
-  </si>
-  <si>
-    <t>REG-054</t>
-  </si>
-  <si>
-    <t>Spaces only in last name</t>
-  </si>
-  <si>
-    <t>aswin.reg054@shopease.com</t>
-  </si>
-  <si>
-    <t>REG-055</t>
-  </si>
-  <si>
-    <t>Spaces only in email</t>
-  </si>
-  <si>
-    <t>REG-056</t>
-  </si>
-  <si>
-    <t>Browser refresh after entering data</t>
-  </si>
-  <si>
-    <t>aswin.reg056@shopease.com</t>
-  </si>
-  <si>
-    <t>STATE HANDLING</t>
-  </si>
-  <si>
-    <t>REG-057</t>
-  </si>
-  <si>
-    <t>Registration after failed attempt</t>
-  </si>
-  <si>
-    <t>aswin.reg057@shopease.com</t>
   </si>
   <si>
     <t>REG-058</t>
@@ -1162,7 +1204,7 @@
         <v>14</v>
       </c>
       <c r="F2">
-        <v>9876543210</v>
+        <v>9123456780</v>
       </c>
       <c r="G2" t="s">
         <v>15</v>
@@ -1185,19 +1227,22 @@
         <v>19</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="D3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
+      </c>
+      <c r="F3">
+        <v>9123456781</v>
       </c>
       <c r="G3" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="H3" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="I3" t="s">
         <v>16</v>
@@ -1208,888 +1253,924 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="C4" t="s">
+        <v>26</v>
       </c>
       <c r="D4" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="F4">
-        <v>9876543210</v>
+        <v>9123456782</v>
       </c>
       <c r="G4" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="H4" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="I4" t="s">
         <v>16</v>
       </c>
       <c r="J4" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C5" t="s">
-        <v>12</v>
+        <v>32</v>
+      </c>
+      <c r="D5" t="s">
+        <v>33</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="F5">
-        <v>9876543210</v>
+        <v>9123456783</v>
       </c>
       <c r="G5" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H5" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I5" t="s">
         <v>16</v>
       </c>
       <c r="J5" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="B6" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="D6" t="s">
-        <v>13</v>
+        <v>40</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>41</v>
       </c>
       <c r="F6">
-        <v>9876543210</v>
+        <v>9123456784</v>
       </c>
       <c r="G6" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H6" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I6" t="s">
         <v>16</v>
       </c>
       <c r="J6" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="B7" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="C7" t="s">
-        <v>12</v>
+        <v>44</v>
       </c>
       <c r="D7" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="F7">
-        <v>9876543210</v>
+        <v>9123456785</v>
+      </c>
+      <c r="G7" t="s">
+        <v>35</v>
+      </c>
+      <c r="H7" t="s">
+        <v>35</v>
       </c>
       <c r="I7" t="s">
         <v>16</v>
       </c>
       <c r="J7" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="B8" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="C8" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="D8" t="s">
-        <v>13</v>
+        <v>48</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="F8">
-        <v>9876543210</v>
+        <v>9123456786</v>
       </c>
       <c r="G8" t="s">
-        <v>15</v>
+        <v>35</v>
+      </c>
+      <c r="H8" t="s">
+        <v>35</v>
       </c>
       <c r="I8" t="s">
         <v>16</v>
       </c>
       <c r="J8" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="B9" t="s">
-        <v>37</v>
+        <v>51</v>
+      </c>
+      <c r="C9" t="s">
+        <v>52</v>
+      </c>
+      <c r="D9" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F9">
+        <v>9123456787</v>
+      </c>
+      <c r="G9" t="s">
+        <v>35</v>
+      </c>
+      <c r="H9" t="s">
+        <v>35</v>
       </c>
       <c r="I9" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="J9" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>39</v>
+        <v>55</v>
       </c>
       <c r="B10" t="s">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="C10" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="D10" t="s">
         <v>13</v>
       </c>
-      <c r="E10" t="s">
-        <v>41</v>
+      <c r="E10" s="2" t="s">
+        <v>58</v>
       </c>
       <c r="F10">
-        <v>9876543210</v>
+        <v>9123456788</v>
       </c>
       <c r="G10" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H10" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I10" t="s">
         <v>16</v>
       </c>
       <c r="J10" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="B11" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="C11" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="D11" t="s">
-        <v>13</v>
-      </c>
-      <c r="E11" t="s">
-        <v>44</v>
+        <v>61</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>62</v>
       </c>
       <c r="F11">
-        <v>9876543210</v>
+        <v>9123456789</v>
       </c>
       <c r="G11" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H11" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I11" t="s">
         <v>16</v>
       </c>
       <c r="J11" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c r="B12" t="s">
-        <v>46</v>
+        <v>64</v>
       </c>
       <c r="C12" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="D12" t="s">
         <v>13</v>
       </c>
-      <c r="E12" t="s">
-        <v>47</v>
+      <c r="E12" s="2" t="s">
+        <v>65</v>
       </c>
       <c r="F12">
-        <v>9876543210</v>
+        <v>9123456790</v>
       </c>
       <c r="G12" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H12" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I12" t="s">
         <v>16</v>
       </c>
       <c r="J12" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>48</v>
+        <v>66</v>
       </c>
       <c r="B13" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="C13" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="D13" t="s">
         <v>13</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="F13">
-        <v>9876543210</v>
+        <v>9123456791</v>
       </c>
       <c r="G13" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H13" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I13" t="s">
         <v>16</v>
       </c>
       <c r="J13" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>51</v>
+        <v>69</v>
       </c>
       <c r="B14" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="C14" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="D14" t="s">
         <v>13</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="F14">
-        <v>9876543210</v>
+        <v>9123456792</v>
       </c>
       <c r="G14" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H14" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I14" t="s">
         <v>16</v>
       </c>
       <c r="J14" t="s">
-        <v>54</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="B15" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="C15" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="D15" t="s">
         <v>13</v>
       </c>
-      <c r="E15" t="s">
-        <v>57</v>
+      <c r="E15" s="2" t="s">
+        <v>75</v>
       </c>
       <c r="F15">
-        <v>9876543210</v>
+        <v>9123456793</v>
       </c>
       <c r="G15" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H15" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I15" t="s">
         <v>16</v>
       </c>
       <c r="J15" t="s">
-        <v>58</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
-        <v>59</v>
+        <v>76</v>
       </c>
       <c r="B16" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="C16" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="D16" t="s">
         <v>13</v>
       </c>
-      <c r="E16" t="s">
-        <v>61</v>
+      <c r="E16" s="2" t="s">
+        <v>78</v>
       </c>
       <c r="F16">
-        <v>9876543210</v>
+        <v>9123456794</v>
       </c>
       <c r="G16" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H16" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I16" t="s">
         <v>16</v>
       </c>
       <c r="J16" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
     </row>
     <row r="17" spans="1:10">
       <c r="A17" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="B17" t="s">
-        <v>63</v>
+        <v>80</v>
       </c>
       <c r="C17" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="D17" t="s">
         <v>13</v>
       </c>
-      <c r="E17" s="2" t="s">
-        <v>64</v>
+      <c r="E17" t="s">
+        <v>81</v>
       </c>
       <c r="F17">
-        <v>9876543210</v>
+        <v>9123456795</v>
       </c>
       <c r="G17" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H17" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I17" t="s">
         <v>16</v>
       </c>
       <c r="J17" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
     </row>
     <row r="18" spans="1:10">
       <c r="A18" t="s">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="B18" t="s">
-        <v>67</v>
+        <v>83</v>
       </c>
       <c r="C18" t="s">
-        <v>68</v>
+        <v>39</v>
       </c>
       <c r="D18" t="s">
-        <v>69</v>
+        <v>13</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>64</v>
+        <v>84</v>
       </c>
       <c r="F18">
-        <v>8765432109</v>
+        <v>9123456796</v>
       </c>
       <c r="G18" t="s">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="H18" t="s">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="I18" t="s">
         <v>16</v>
       </c>
       <c r="J18" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="B19" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="C19" t="s">
-        <v>68</v>
+        <v>39</v>
       </c>
       <c r="D19" t="s">
-        <v>69</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>64</v>
+        <v>13</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>87</v>
       </c>
       <c r="F19">
-        <v>8765432109</v>
+        <v>9123456797</v>
       </c>
       <c r="G19" t="s">
-        <v>73</v>
+        <v>35</v>
       </c>
       <c r="H19" t="s">
-        <v>73</v>
+        <v>35</v>
       </c>
       <c r="I19" t="s">
         <v>16</v>
       </c>
       <c r="J19" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="B20" t="s">
-        <v>75</v>
+        <v>89</v>
       </c>
       <c r="C20" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="D20" t="s">
         <v>13</v>
       </c>
-      <c r="E20" s="2" t="s">
-        <v>76</v>
+      <c r="E20" t="s">
+        <v>90</v>
       </c>
       <c r="F20">
-        <v>9876543210</v>
+        <v>9123456798</v>
       </c>
       <c r="G20" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H20" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I20" t="s">
         <v>16</v>
       </c>
       <c r="J20" t="s">
-        <v>17</v>
+        <v>54</v>
       </c>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" t="s">
-        <v>77</v>
+        <v>91</v>
       </c>
       <c r="B21" t="s">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="C21" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="D21" t="s">
         <v>13</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>79</v>
+        <v>93</v>
       </c>
       <c r="F21">
-        <v>9876543210</v>
+        <v>9123456799</v>
       </c>
       <c r="G21" t="s">
-        <v>15</v>
+        <v>94</v>
       </c>
       <c r="H21" t="s">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="I21" t="s">
         <v>16</v>
       </c>
       <c r="J21" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
     </row>
     <row r="22" spans="1:10">
       <c r="A22" t="s">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="B22" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="C22" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="D22" t="s">
         <v>13</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>83</v>
+        <v>97</v>
       </c>
       <c r="F22">
-        <v>9876543210</v>
+        <v>9123456800</v>
       </c>
       <c r="G22" t="s">
-        <v>15</v>
+        <v>98</v>
       </c>
       <c r="H22" t="s">
-        <v>84</v>
+        <v>98</v>
       </c>
       <c r="I22" t="s">
         <v>16</v>
       </c>
       <c r="J22" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
     </row>
     <row r="23" spans="1:10">
       <c r="A23" t="s">
-        <v>85</v>
+        <v>99</v>
       </c>
       <c r="B23" t="s">
-        <v>86</v>
+        <v>100</v>
       </c>
       <c r="C23" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="D23" t="s">
         <v>13</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="F23">
-        <v>9876543210</v>
+        <v>9123456801</v>
       </c>
       <c r="G23" t="s">
-        <v>15</v>
+        <v>102</v>
       </c>
       <c r="H23" t="s">
-        <v>88</v>
+        <v>102</v>
       </c>
       <c r="I23" t="s">
         <v>16</v>
       </c>
       <c r="J23" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
     </row>
     <row r="24" spans="1:10">
       <c r="A24" t="s">
-        <v>89</v>
+        <v>103</v>
       </c>
       <c r="B24" t="s">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="C24" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="D24" t="s">
         <v>13</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>91</v>
+        <v>105</v>
       </c>
       <c r="F24">
-        <v>9876543210</v>
+        <v>9123456802</v>
       </c>
       <c r="G24" t="s">
-        <v>92</v>
+        <v>35</v>
       </c>
       <c r="H24" t="s">
-        <v>92</v>
+        <v>35</v>
       </c>
       <c r="I24" t="s">
         <v>16</v>
       </c>
       <c r="J24" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
     </row>
     <row r="25" spans="1:10">
       <c r="A25" t="s">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="B25" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="C25" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="D25" t="s">
         <v>13</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="F25">
-        <v>9876543210</v>
+        <v>9123456803</v>
       </c>
       <c r="G25" t="s">
-        <v>96</v>
+        <v>35</v>
       </c>
       <c r="H25" t="s">
-        <v>96</v>
+        <v>35</v>
       </c>
       <c r="I25" t="s">
         <v>16</v>
       </c>
       <c r="J25" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
     </row>
     <row r="26" spans="1:10">
       <c r="A26" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="B26" t="s">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="C26" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="D26" t="s">
         <v>13</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>99</v>
+        <v>111</v>
       </c>
       <c r="F26">
-        <v>9876543210</v>
-      </c>
-      <c r="G26">
-        <v>123456</v>
-      </c>
-      <c r="H26">
-        <v>123456</v>
+        <v>9123456804</v>
+      </c>
+      <c r="G26" t="s">
+        <v>35</v>
+      </c>
+      <c r="H26" t="s">
+        <v>35</v>
       </c>
       <c r="I26" t="s">
         <v>16</v>
       </c>
       <c r="J26" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="27" spans="1:10">
       <c r="A27" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="B27" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
       <c r="C27" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="D27" t="s">
         <v>13</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="F27">
-        <v>9876543210</v>
+        <v>9123456805</v>
       </c>
       <c r="G27" t="s">
-        <v>103</v>
+        <v>35</v>
       </c>
       <c r="H27" t="s">
-        <v>103</v>
+        <v>35</v>
       </c>
       <c r="I27" t="s">
         <v>16</v>
       </c>
       <c r="J27" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="28" spans="1:10">
       <c r="A28" t="s">
-        <v>104</v>
+        <v>115</v>
       </c>
       <c r="B28" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
       <c r="C28" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="D28" t="s">
         <v>13</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="F28">
-        <v>9876543210</v>
-      </c>
-      <c r="G28" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="H28" s="3" t="s">
-        <v>107</v>
+        <v>987654321</v>
+      </c>
+      <c r="G28" t="s">
+        <v>35</v>
+      </c>
+      <c r="H28" t="s">
+        <v>35</v>
       </c>
       <c r="I28" t="s">
         <v>16</v>
       </c>
       <c r="J28" t="s">
-        <v>58</v>
+        <v>118</v>
       </c>
     </row>
     <row r="29" spans="1:10">
       <c r="A29" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
       <c r="B29" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
       <c r="C29" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="D29" t="s">
         <v>13</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="F29">
-        <v>9876543210</v>
+        <v>121</v>
+      </c>
+      <c r="F29" t="s">
+        <v>122</v>
       </c>
       <c r="G29" t="s">
-        <v>111</v>
+        <v>35</v>
       </c>
       <c r="H29" t="s">
-        <v>111</v>
+        <v>35</v>
       </c>
       <c r="I29" t="s">
         <v>16</v>
       </c>
       <c r="J29" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="30" spans="1:10">
       <c r="A30" t="s">
-        <v>112</v>
+        <v>123</v>
       </c>
       <c r="B30" t="s">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="C30" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="D30" t="s">
         <v>13</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>114</v>
+        <v>125</v>
       </c>
       <c r="F30">
-        <v>9876543210</v>
+        <v>919876543210</v>
       </c>
       <c r="G30" t="s">
-        <v>115</v>
+        <v>35</v>
       </c>
       <c r="H30" t="s">
-        <v>115</v>
+        <v>35</v>
       </c>
       <c r="I30" t="s">
         <v>16</v>
       </c>
       <c r="J30" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="B31" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="C31" t="s">
-        <v>12</v>
+        <v>128</v>
       </c>
       <c r="D31" t="s">
-        <v>13</v>
+        <v>129</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>118</v>
+        <v>130</v>
       </c>
       <c r="F31">
-        <v>9876543210</v>
+        <v>9123456810</v>
       </c>
       <c r="G31" t="s">
-        <v>15</v>
+        <v>131</v>
       </c>
       <c r="H31" t="s">
-        <v>15</v>
+        <v>131</v>
       </c>
       <c r="I31" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="J31" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="B32" t="s">
-        <v>120</v>
+        <v>133</v>
       </c>
       <c r="C32" t="s">
-        <v>12</v>
+        <v>134</v>
       </c>
       <c r="D32" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="F32">
         <v>9876543210</v>
       </c>
       <c r="G32" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H32" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I32" t="s">
         <v>16</v>
@@ -2100,252 +2181,252 @@
     </row>
     <row r="33" spans="1:10">
       <c r="A33" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
       <c r="B33" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
       <c r="C33" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="D33" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="F33">
         <v>9876543210</v>
       </c>
       <c r="G33" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H33" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I33" t="s">
         <v>16</v>
       </c>
       <c r="J33" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
     </row>
     <row r="34" spans="1:10">
       <c r="A34" t="s">
-        <v>127</v>
+        <v>141</v>
       </c>
       <c r="B34" t="s">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="C34" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="D34" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
       <c r="F34">
         <v>9876543210</v>
       </c>
       <c r="G34" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H34" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I34" t="s">
         <v>16</v>
       </c>
       <c r="J34" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
     </row>
     <row r="35" spans="1:10">
       <c r="A35" t="s">
-        <v>131</v>
+        <v>145</v>
       </c>
       <c r="B35" t="s">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="C35" t="s">
-        <v>12</v>
+        <v>134</v>
       </c>
       <c r="D35" t="s">
-        <v>133</v>
+        <v>147</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>134</v>
+        <v>148</v>
       </c>
       <c r="F35">
         <v>9876543210</v>
       </c>
       <c r="G35" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H35" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I35" t="s">
         <v>16</v>
       </c>
       <c r="J35" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
     </row>
     <row r="36" spans="1:10">
       <c r="A36" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
       <c r="B36" t="s">
-        <v>136</v>
+        <v>150</v>
       </c>
       <c r="C36" t="s">
-        <v>137</v>
+        <v>151</v>
       </c>
       <c r="D36" t="s">
-        <v>138</v>
+        <v>33</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>139</v>
+        <v>152</v>
       </c>
       <c r="F36">
         <v>9876543210</v>
       </c>
       <c r="G36" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H36" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I36" t="s">
         <v>16</v>
       </c>
       <c r="J36" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
     </row>
     <row r="37" spans="1:10">
       <c r="A37" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
       <c r="B37" t="s">
-        <v>141</v>
+        <v>154</v>
       </c>
       <c r="C37" t="s">
-        <v>142</v>
+        <v>155</v>
       </c>
       <c r="D37" t="s">
-        <v>138</v>
+        <v>33</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>143</v>
+        <v>156</v>
       </c>
       <c r="F37">
         <v>9876543210</v>
       </c>
       <c r="G37" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H37" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I37" t="s">
         <v>16</v>
       </c>
       <c r="J37" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
     </row>
     <row r="38" spans="1:10">
       <c r="A38" t="s">
-        <v>144</v>
+        <v>157</v>
       </c>
       <c r="B38" t="s">
-        <v>145</v>
+        <v>158</v>
       </c>
       <c r="C38" t="s">
-        <v>146</v>
+        <v>159</v>
       </c>
       <c r="D38" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="F38">
         <v>9876543210</v>
       </c>
       <c r="G38" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H38" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I38" t="s">
         <v>16</v>
       </c>
       <c r="J38" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
     </row>
     <row r="39" spans="1:10">
       <c r="A39" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="B39" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="C39" t="s">
-        <v>12</v>
+        <v>134</v>
       </c>
       <c r="D39" t="s">
-        <v>150</v>
+        <v>163</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>151</v>
+        <v>164</v>
       </c>
       <c r="F39">
         <v>9876543210</v>
       </c>
       <c r="G39" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H39" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I39" t="s">
         <v>16</v>
       </c>
       <c r="J39" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
     </row>
     <row r="40" spans="1:10">
       <c r="A40" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="B40" t="s">
-        <v>153</v>
+        <v>166</v>
       </c>
       <c r="C40" t="s">
-        <v>12</v>
+        <v>134</v>
       </c>
       <c r="D40" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>154</v>
+        <v>167</v>
       </c>
       <c r="F40">
         <v>9876543210</v>
       </c>
       <c r="G40" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H40" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I40" t="s">
         <v>16</v>
@@ -2356,595 +2437,595 @@
     </row>
     <row r="41" spans="1:10">
       <c r="A41" t="s">
-        <v>155</v>
+        <v>168</v>
       </c>
       <c r="B41" t="s">
-        <v>156</v>
+        <v>169</v>
       </c>
       <c r="C41" t="s">
-        <v>12</v>
+        <v>134</v>
       </c>
       <c r="D41" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>157</v>
+        <v>170</v>
       </c>
       <c r="F41">
         <v>987654321</v>
       </c>
       <c r="G41" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H41" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I41" t="s">
         <v>16</v>
       </c>
       <c r="J41" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
     </row>
     <row r="42" spans="1:10">
       <c r="A42" t="s">
-        <v>158</v>
+        <v>171</v>
       </c>
       <c r="B42" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="C42" t="s">
-        <v>12</v>
+        <v>134</v>
       </c>
       <c r="D42" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="F42">
         <v>98765432101</v>
       </c>
       <c r="G42" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H42" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I42" t="s">
         <v>16</v>
       </c>
       <c r="J42" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
     </row>
     <row r="43" spans="1:10">
       <c r="A43" t="s">
-        <v>161</v>
+        <v>174</v>
       </c>
       <c r="B43" t="s">
-        <v>162</v>
+        <v>175</v>
       </c>
       <c r="C43" t="s">
-        <v>12</v>
+        <v>134</v>
       </c>
       <c r="D43" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>163</v>
+        <v>176</v>
       </c>
       <c r="F43" t="s">
-        <v>164</v>
+        <v>177</v>
       </c>
       <c r="G43" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H43" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I43" t="s">
         <v>16</v>
       </c>
       <c r="J43" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
     </row>
     <row r="44" spans="1:10">
       <c r="A44" t="s">
-        <v>165</v>
+        <v>178</v>
       </c>
       <c r="B44" t="s">
-        <v>166</v>
+        <v>179</v>
       </c>
       <c r="C44" t="s">
-        <v>12</v>
+        <v>134</v>
       </c>
       <c r="D44" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="F44" t="s">
-        <v>168</v>
+        <v>181</v>
       </c>
       <c r="G44" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H44" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I44" t="s">
         <v>16</v>
       </c>
       <c r="J44" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
     </row>
     <row r="45" spans="1:10">
       <c r="A45" t="s">
-        <v>169</v>
+        <v>182</v>
       </c>
       <c r="B45" t="s">
-        <v>170</v>
+        <v>183</v>
       </c>
       <c r="C45" t="s">
-        <v>12</v>
+        <v>134</v>
       </c>
       <c r="D45" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>171</v>
+        <v>184</v>
       </c>
       <c r="F45">
         <v>919876543210</v>
       </c>
       <c r="G45" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H45" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I45" t="s">
         <v>16</v>
       </c>
       <c r="J45" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
     </row>
     <row r="46" spans="1:10">
       <c r="A46" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="B46" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="C46" t="s">
-        <v>12</v>
+        <v>134</v>
       </c>
       <c r="D46" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
       <c r="F46">
         <v>0</v>
       </c>
       <c r="G46" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H46" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I46" t="s">
         <v>16</v>
       </c>
       <c r="J46" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
     </row>
     <row r="47" spans="1:10">
       <c r="A47" t="s">
-        <v>175</v>
+        <v>188</v>
       </c>
       <c r="B47" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="C47" t="s">
-        <v>12</v>
+        <v>134</v>
       </c>
       <c r="D47" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>177</v>
+        <v>190</v>
       </c>
       <c r="F47">
         <v>9876543210</v>
       </c>
       <c r="G47" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H47" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I47" t="s">
         <v>16</v>
       </c>
       <c r="J47" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
     </row>
     <row r="48" spans="1:10">
       <c r="A48" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
       <c r="B48" t="s">
-        <v>179</v>
+        <v>192</v>
       </c>
       <c r="C48" t="s">
-        <v>12</v>
+        <v>134</v>
       </c>
       <c r="D48" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
       <c r="F48">
         <v>9876543210</v>
       </c>
       <c r="G48" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H48" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I48" t="s">
         <v>16</v>
       </c>
       <c r="J48" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
     </row>
     <row r="49" spans="1:10">
       <c r="A49" t="s">
-        <v>181</v>
+        <v>194</v>
       </c>
       <c r="B49" t="s">
-        <v>182</v>
+        <v>195</v>
       </c>
       <c r="C49" t="s">
-        <v>12</v>
+        <v>134</v>
       </c>
       <c r="D49" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>183</v>
+        <v>196</v>
       </c>
       <c r="F49">
         <v>9876543210</v>
       </c>
       <c r="G49" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H49" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I49" t="s">
         <v>16</v>
       </c>
       <c r="J49" t="s">
-        <v>184</v>
+        <v>197</v>
       </c>
     </row>
     <row r="50" spans="1:10">
       <c r="A50" t="s">
-        <v>185</v>
+        <v>198</v>
       </c>
       <c r="B50" t="s">
-        <v>186</v>
+        <v>199</v>
       </c>
       <c r="C50" t="s">
-        <v>12</v>
+        <v>134</v>
       </c>
       <c r="D50" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="F50">
         <v>9876543210</v>
       </c>
       <c r="G50" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H50" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I50" t="s">
         <v>16</v>
       </c>
       <c r="J50" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
     </row>
     <row r="51" spans="1:10">
       <c r="A51" t="s">
-        <v>189</v>
+        <v>202</v>
       </c>
       <c r="B51" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="D51" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="F51">
         <v>9876543210</v>
       </c>
       <c r="G51" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H51" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I51" t="s">
         <v>16</v>
       </c>
       <c r="J51" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
     </row>
     <row r="52" spans="1:10">
       <c r="A52" t="s">
-        <v>194</v>
+        <v>207</v>
       </c>
       <c r="B52" t="s">
-        <v>195</v>
+        <v>208</v>
       </c>
       <c r="C52" t="s">
-        <v>196</v>
+        <v>209</v>
       </c>
       <c r="D52" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>197</v>
+        <v>210</v>
       </c>
       <c r="F52">
         <v>9876543210</v>
       </c>
       <c r="G52" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H52" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I52" t="s">
         <v>16</v>
       </c>
       <c r="J52" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
     </row>
     <row r="53" spans="1:10">
       <c r="A53" t="s">
-        <v>198</v>
+        <v>211</v>
       </c>
       <c r="B53" t="s">
-        <v>199</v>
+        <v>212</v>
       </c>
       <c r="C53" t="s">
-        <v>12</v>
+        <v>134</v>
       </c>
       <c r="D53" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E53" t="s">
-        <v>196</v>
+        <v>209</v>
       </c>
       <c r="F53">
         <v>9876543210</v>
       </c>
       <c r="G53" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H53" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I53" t="s">
         <v>16</v>
       </c>
       <c r="J53" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
     </row>
     <row r="54" spans="1:10">
       <c r="A54" t="s">
-        <v>200</v>
+        <v>213</v>
       </c>
       <c r="B54" t="s">
-        <v>201</v>
+        <v>214</v>
       </c>
       <c r="D54" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>202</v>
+        <v>215</v>
       </c>
       <c r="F54">
         <v>9876543210</v>
       </c>
       <c r="G54" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H54" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I54" t="s">
         <v>16</v>
       </c>
       <c r="J54" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
     </row>
     <row r="55" spans="1:10">
       <c r="A55" t="s">
-        <v>203</v>
+        <v>216</v>
       </c>
       <c r="B55" t="s">
-        <v>204</v>
+        <v>217</v>
       </c>
       <c r="C55" t="s">
-        <v>12</v>
+        <v>134</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>205</v>
+        <v>218</v>
       </c>
       <c r="F55">
         <v>9876543210</v>
       </c>
       <c r="G55" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H55" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I55" t="s">
         <v>16</v>
       </c>
       <c r="J55" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
     </row>
     <row r="56" spans="1:10">
       <c r="A56" t="s">
-        <v>206</v>
+        <v>219</v>
       </c>
       <c r="B56" t="s">
-        <v>207</v>
+        <v>220</v>
       </c>
       <c r="C56" t="s">
-        <v>12</v>
+        <v>134</v>
       </c>
       <c r="D56" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="F56">
         <v>9876543210</v>
       </c>
       <c r="G56" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H56" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I56" t="s">
         <v>16</v>
       </c>
       <c r="J56" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
     </row>
     <row r="57" spans="1:10">
       <c r="A57" t="s">
-        <v>208</v>
+        <v>221</v>
       </c>
       <c r="B57" t="s">
-        <v>209</v>
+        <v>222</v>
       </c>
       <c r="C57" t="s">
-        <v>12</v>
+        <v>134</v>
       </c>
       <c r="D57" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>210</v>
+        <v>223</v>
       </c>
       <c r="F57">
         <v>9876543210</v>
       </c>
       <c r="G57" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H57" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I57" t="s">
         <v>16</v>
       </c>
       <c r="J57" t="s">
-        <v>211</v>
+        <v>224</v>
       </c>
     </row>
     <row r="58" spans="1:10">
       <c r="A58" t="s">
-        <v>212</v>
+        <v>225</v>
       </c>
       <c r="B58" t="s">
-        <v>213</v>
+        <v>226</v>
       </c>
       <c r="C58" t="s">
-        <v>12</v>
+        <v>134</v>
       </c>
       <c r="D58" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>214</v>
+        <v>227</v>
       </c>
       <c r="F58">
         <v>9876543210</v>
       </c>
       <c r="G58" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H58" t="s">
-        <v>80</v>
+        <v>228</v>
       </c>
       <c r="I58" t="s">
         <v>16</v>
       </c>
       <c r="J58" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
     </row>
     <row r="59" spans="1:10">
       <c r="A59" t="s">
-        <v>215</v>
+        <v>229</v>
       </c>
       <c r="B59" t="s">
-        <v>216</v>
+        <v>230</v>
       </c>
       <c r="C59" t="s">
-        <v>12</v>
+        <v>134</v>
       </c>
       <c r="D59" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>217</v>
+        <v>231</v>
       </c>
       <c r="F59">
         <v>9876543210</v>
       </c>
       <c r="G59" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H59" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I59" t="s">
         <v>16</v>
@@ -2955,60 +3036,60 @@
     </row>
     <row r="60" spans="1:10">
       <c r="A60" t="s">
-        <v>218</v>
+        <v>232</v>
       </c>
       <c r="B60" t="s">
-        <v>219</v>
+        <v>233</v>
       </c>
       <c r="C60" t="s">
-        <v>12</v>
+        <v>134</v>
       </c>
       <c r="D60" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>220</v>
+        <v>234</v>
       </c>
       <c r="F60">
         <v>9876543210</v>
       </c>
       <c r="G60" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H60" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I60" t="s">
         <v>16</v>
       </c>
       <c r="J60" t="s">
-        <v>221</v>
+        <v>235</v>
       </c>
     </row>
     <row r="61" spans="1:10">
       <c r="A61" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="B61" t="s">
-        <v>223</v>
+        <v>237</v>
       </c>
       <c r="C61" t="s">
-        <v>12</v>
+        <v>134</v>
       </c>
       <c r="D61" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>224</v>
+        <v>238</v>
       </c>
       <c r="F61">
         <v>9876543210</v>
       </c>
       <c r="G61" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H61" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="I61" t="s">
         <v>16</v>
@@ -3019,57 +3100,61 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1" xr:uid="{E8754A02-F45B-4A0E-950A-235A9F78ADF9}"/>
-    <hyperlink ref="E3" r:id="rId2" xr:uid="{ECE16905-1131-4177-897C-B8A4C6FE41A8}"/>
-    <hyperlink ref="E4" r:id="rId3" xr:uid="{AD2076DF-56C6-4058-87B1-331A5EFCAD3D}"/>
-    <hyperlink ref="E5" r:id="rId4" xr:uid="{E852D243-5F59-4FF9-A1E2-E546E3FE2D59}"/>
-    <hyperlink ref="E7" r:id="rId5" xr:uid="{FA425C20-C0ED-4675-9603-6693D2DB1467}"/>
-    <hyperlink ref="E8" r:id="rId6" xr:uid="{3E9357B8-11BC-4ADC-9975-2FCC406FA531}"/>
-    <hyperlink ref="E13" r:id="rId7" xr:uid="{56D4DBC2-249A-47D2-97D8-CC4F94865409}"/>
-    <hyperlink ref="E14" r:id="rId8" xr:uid="{9EC59D41-5C8F-4B24-BDA9-B403CA5D80AB}"/>
-    <hyperlink ref="E17" r:id="rId9" xr:uid="{ECEA5928-6B06-4A8E-80DD-76116DD419DB}"/>
-    <hyperlink ref="E18" r:id="rId10" xr:uid="{9D4988B8-F29E-4D72-88CA-580C18CDD710}"/>
-    <hyperlink ref="E19" r:id="rId11" xr:uid="{4528BD2E-BB12-412E-8DDD-BAC802384B8B}"/>
-    <hyperlink ref="E20" r:id="rId12" xr:uid="{D2E97D42-5388-4DCC-BB41-126542296CBB}"/>
-    <hyperlink ref="E21" r:id="rId13" xr:uid="{BF4E494E-6BD7-4214-BFC9-EFC86ED1DA32}"/>
-    <hyperlink ref="E22" r:id="rId14" xr:uid="{C7CD9767-55D9-4518-8A17-92EF0153B349}"/>
-    <hyperlink ref="E23" r:id="rId15" xr:uid="{6FE4853B-D27A-442A-8E41-42BE6EB238C5}"/>
-    <hyperlink ref="E24" r:id="rId16" xr:uid="{1D5C93E8-1144-48F6-9526-F195EB7297C0}"/>
-    <hyperlink ref="E25" r:id="rId17" xr:uid="{32C9A16E-CEE9-4859-BA2D-F133C5AADA97}"/>
-    <hyperlink ref="E26" r:id="rId18" xr:uid="{1AA75202-9B32-48A5-A214-56B6A7E51E99}"/>
-    <hyperlink ref="E27" r:id="rId19" xr:uid="{33453737-9D4C-4372-9C3C-186480DD572F}"/>
-    <hyperlink ref="E28" r:id="rId20" xr:uid="{17529BDA-6CF6-4932-9E28-7E32F8974D3A}"/>
-    <hyperlink ref="E29" r:id="rId21" xr:uid="{9A76FF4C-AFB2-4012-8BA1-8E9C8AABC53F}"/>
-    <hyperlink ref="E30" r:id="rId22" xr:uid="{30C01598-AC18-4E00-8A22-C91D855A7C84}"/>
-    <hyperlink ref="E31" r:id="rId23" xr:uid="{7CB5158D-4D17-4CE6-BDA6-2B0205D47E27}"/>
-    <hyperlink ref="E32" r:id="rId24" xr:uid="{00D45D92-B13E-4FB8-8AE3-A59C76E391BD}"/>
-    <hyperlink ref="E33" r:id="rId25" xr:uid="{3C213E58-5C55-4727-8E88-BD6DA63D7889}"/>
-    <hyperlink ref="E34" r:id="rId26" xr:uid="{AE071C29-A25E-4B5A-97DD-7CA75E42AC43}"/>
-    <hyperlink ref="E35" r:id="rId27" xr:uid="{B0D14CEF-60F1-426B-AA0C-AA837D3751A6}"/>
-    <hyperlink ref="E36" r:id="rId28" xr:uid="{70A4705A-56CD-47EE-8A3E-6D9F8F3E163B}"/>
-    <hyperlink ref="E37" r:id="rId29" xr:uid="{65F37F58-43B7-43FC-92ED-29C905790D07}"/>
-    <hyperlink ref="E38" r:id="rId30" xr:uid="{D166FDBE-D8DD-4CC7-BBA2-4B09841FE632}"/>
-    <hyperlink ref="E39" r:id="rId31" xr:uid="{72EAFAC9-9E7B-4F20-8C67-7F52396C0634}"/>
-    <hyperlink ref="E40" r:id="rId32" xr:uid="{A531EFCD-9FC9-45F9-A1E4-D510A099A43D}"/>
-    <hyperlink ref="E41" r:id="rId33" xr:uid="{DF473D7F-7988-43C8-B5B4-B19585D8E4F5}"/>
-    <hyperlink ref="E42" r:id="rId34" xr:uid="{E273AF84-0DBB-4DCA-8C26-30CF316BDF42}"/>
-    <hyperlink ref="E43" r:id="rId35" xr:uid="{7438A9D1-D38D-4990-B7DD-7C20823087B4}"/>
-    <hyperlink ref="E44" r:id="rId36" xr:uid="{4EDD6734-F78D-431F-A706-DDC6492887C4}"/>
-    <hyperlink ref="E45" r:id="rId37" xr:uid="{C637B3D0-D25C-4C95-AB0A-CDBDFC8884E2}"/>
-    <hyperlink ref="E46" r:id="rId38" xr:uid="{D5937380-F3D9-4E90-BD55-04212E77D351}"/>
-    <hyperlink ref="E47" r:id="rId39" xr:uid="{443D53F6-5864-41E4-9D5D-55A1763135DC}"/>
-    <hyperlink ref="E48" r:id="rId40" xr:uid="{6C1C1234-D136-4583-9675-0F847A4C3203}"/>
-    <hyperlink ref="E49" r:id="rId41" xr:uid="{15ED420C-C5E7-4B6C-99E5-D697325737D2}"/>
-    <hyperlink ref="E50" r:id="rId42" xr:uid="{D8322BCF-51EC-4607-B700-6AE8AE74E158}"/>
-    <hyperlink ref="E51" r:id="rId43" xr:uid="{47469ECE-EA77-4865-90C2-3179877C3E7A}"/>
-    <hyperlink ref="E52" r:id="rId44" xr:uid="{A913695F-2080-45E0-B7BB-CD11DE79B8CA}"/>
-    <hyperlink ref="E54" r:id="rId45" xr:uid="{D3358117-7D34-4D12-9B19-F25DF0A16902}"/>
-    <hyperlink ref="E55" r:id="rId46" xr:uid="{4E10B0BE-6EB0-49EC-9248-A61657EAAB1B}"/>
-    <hyperlink ref="E57" r:id="rId47" xr:uid="{BF39DA02-BD28-4CDC-9483-35AD286EBDF7}"/>
-    <hyperlink ref="E58" r:id="rId48" xr:uid="{282616F8-6F0B-4BF2-8E32-76C4917BB9A3}"/>
-    <hyperlink ref="E59" r:id="rId49" xr:uid="{E9E0AFC6-87FC-47EA-9595-BD623ACA36E2}"/>
-    <hyperlink ref="E60" r:id="rId50" xr:uid="{136E713D-E2DF-43F9-B35F-546C5EA09B7E}"/>
-    <hyperlink ref="E61" r:id="rId51" xr:uid="{A8207317-6324-4FFD-BF70-D2EA45639663}"/>
+    <hyperlink ref="E32" r:id="rId1" xr:uid="{00D45D92-B13E-4FB8-8AE3-A59C76E391BD}"/>
+    <hyperlink ref="E33" r:id="rId2" xr:uid="{3C213E58-5C55-4727-8E88-BD6DA63D7889}"/>
+    <hyperlink ref="E34" r:id="rId3" xr:uid="{AE071C29-A25E-4B5A-97DD-7CA75E42AC43}"/>
+    <hyperlink ref="E35" r:id="rId4" xr:uid="{B0D14CEF-60F1-426B-AA0C-AA837D3751A6}"/>
+    <hyperlink ref="E36" r:id="rId5" xr:uid="{70A4705A-56CD-47EE-8A3E-6D9F8F3E163B}"/>
+    <hyperlink ref="E37" r:id="rId6" xr:uid="{65F37F58-43B7-43FC-92ED-29C905790D07}"/>
+    <hyperlink ref="E38" r:id="rId7" xr:uid="{D166FDBE-D8DD-4CC7-BBA2-4B09841FE632}"/>
+    <hyperlink ref="E39" r:id="rId8" xr:uid="{72EAFAC9-9E7B-4F20-8C67-7F52396C0634}"/>
+    <hyperlink ref="E40" r:id="rId9" xr:uid="{A531EFCD-9FC9-45F9-A1E4-D510A099A43D}"/>
+    <hyperlink ref="E41" r:id="rId10" xr:uid="{DF473D7F-7988-43C8-B5B4-B19585D8E4F5}"/>
+    <hyperlink ref="E42" r:id="rId11" xr:uid="{E273AF84-0DBB-4DCA-8C26-30CF316BDF42}"/>
+    <hyperlink ref="E43" r:id="rId12" xr:uid="{7438A9D1-D38D-4990-B7DD-7C20823087B4}"/>
+    <hyperlink ref="E44" r:id="rId13" xr:uid="{4EDD6734-F78D-431F-A706-DDC6492887C4}"/>
+    <hyperlink ref="E45" r:id="rId14" xr:uid="{C637B3D0-D25C-4C95-AB0A-CDBDFC8884E2}"/>
+    <hyperlink ref="E46" r:id="rId15" xr:uid="{D5937380-F3D9-4E90-BD55-04212E77D351}"/>
+    <hyperlink ref="E47" r:id="rId16" xr:uid="{443D53F6-5864-41E4-9D5D-55A1763135DC}"/>
+    <hyperlink ref="E48" r:id="rId17" xr:uid="{6C1C1234-D136-4583-9675-0F847A4C3203}"/>
+    <hyperlink ref="E49" r:id="rId18" xr:uid="{15ED420C-C5E7-4B6C-99E5-D697325737D2}"/>
+    <hyperlink ref="E50" r:id="rId19" xr:uid="{D8322BCF-51EC-4607-B700-6AE8AE74E158}"/>
+    <hyperlink ref="E51" r:id="rId20" xr:uid="{47469ECE-EA77-4865-90C2-3179877C3E7A}"/>
+    <hyperlink ref="E52" r:id="rId21" xr:uid="{A913695F-2080-45E0-B7BB-CD11DE79B8CA}"/>
+    <hyperlink ref="E54" r:id="rId22" xr:uid="{D3358117-7D34-4D12-9B19-F25DF0A16902}"/>
+    <hyperlink ref="E55" r:id="rId23" xr:uid="{4E10B0BE-6EB0-49EC-9248-A61657EAAB1B}"/>
+    <hyperlink ref="E57" r:id="rId24" xr:uid="{BF39DA02-BD28-4CDC-9483-35AD286EBDF7}"/>
+    <hyperlink ref="E58" r:id="rId25" xr:uid="{282616F8-6F0B-4BF2-8E32-76C4917BB9A3}"/>
+    <hyperlink ref="E59" r:id="rId26" xr:uid="{E9E0AFC6-87FC-47EA-9595-BD623ACA36E2}"/>
+    <hyperlink ref="E60" r:id="rId27" xr:uid="{136E713D-E2DF-43F9-B35F-546C5EA09B7E}"/>
+    <hyperlink ref="E61" r:id="rId28" xr:uid="{A8207317-6324-4FFD-BF70-D2EA45639663}"/>
+    <hyperlink ref="E2" r:id="rId29" xr:uid="{FA411A1F-4C6C-41AE-9029-07F3EE09C0DF}"/>
+    <hyperlink ref="E3" r:id="rId30" xr:uid="{8D2E4C3B-8774-4D98-9AAC-779F4B084528}"/>
+    <hyperlink ref="E4" r:id="rId31" xr:uid="{F90055E4-8CE2-4C1C-ABC5-121C7555A9EC}"/>
+    <hyperlink ref="E5" r:id="rId32" xr:uid="{ED4E0E1A-A541-494F-AD1E-E0EB7A44622C}"/>
+    <hyperlink ref="E6" r:id="rId33" xr:uid="{10737B0C-526C-4E59-A6EA-3CBEF89895C2}"/>
+    <hyperlink ref="E7" r:id="rId34" xr:uid="{D42AAF2E-2327-42C5-BF30-47D5E8705935}"/>
+    <hyperlink ref="E8" r:id="rId35" xr:uid="{79E78683-C376-48CF-8963-766092F3A4BA}"/>
+    <hyperlink ref="E9" r:id="rId36" xr:uid="{1D758152-98A8-4EFC-826D-39A8E4F0C5D6}"/>
+    <hyperlink ref="E10" r:id="rId37" xr:uid="{55DEB8F3-7046-4FCB-B82B-1A62EBE69020}"/>
+    <hyperlink ref="E11" r:id="rId38" xr:uid="{3B7C50C8-B327-4450-BC1C-DC4076210591}"/>
+    <hyperlink ref="E12" r:id="rId39" xr:uid="{7689D2F1-7567-49F9-8015-14AEA64A7A21}"/>
+    <hyperlink ref="E13" r:id="rId40" xr:uid="{B4F4B65D-105C-45BE-B9DC-6207FEC98FD6}"/>
+    <hyperlink ref="E14" r:id="rId41" xr:uid="{3F34AE4F-2B87-4504-BF1A-03D4A065F218}"/>
+    <hyperlink ref="E15" r:id="rId42" xr:uid="{01E1FF33-750D-4727-B7A2-236E70E21817}"/>
+    <hyperlink ref="E16" r:id="rId43" xr:uid="{DE867148-4E5B-4DF4-8F4A-9AF4013C603C}"/>
+    <hyperlink ref="E18" r:id="rId44" xr:uid="{D1ACE657-1B61-4412-8A82-BEADA4E5B47F}"/>
+    <hyperlink ref="E21" r:id="rId45" xr:uid="{8AE521B6-18D1-4B42-BD01-53E954C0A6E7}"/>
+    <hyperlink ref="E22" r:id="rId46" xr:uid="{740E425D-1F0B-447C-8E3B-0D3E9F80491B}"/>
+    <hyperlink ref="E23" r:id="rId47" xr:uid="{F7495715-9ED6-4B52-B63E-79DB1671E997}"/>
+    <hyperlink ref="E24" r:id="rId48" xr:uid="{F502D8DC-A3F3-4834-86CC-6E5B3BD2CF79}"/>
+    <hyperlink ref="E25" r:id="rId49" xr:uid="{88BB17D7-8DAC-4032-88DC-C8DAE0A52298}"/>
+    <hyperlink ref="E26" r:id="rId50" xr:uid="{9A30E1CB-A740-4EF3-80AB-76CE90CBB2A1}"/>
+    <hyperlink ref="E27" r:id="rId51" xr:uid="{29B8BA89-E2E8-4948-81A6-5E90D61BD972}"/>
+    <hyperlink ref="E28" r:id="rId52" xr:uid="{AA0EA52A-4B97-48AE-9191-8DF20D0F2E9D}"/>
+    <hyperlink ref="E29" r:id="rId53" xr:uid="{686E9826-B31E-4222-B036-1A6A9D9A7F80}"/>
+    <hyperlink ref="E30" r:id="rId54" xr:uid="{13185B49-302E-4E72-A91F-D246D40A8254}"/>
+    <hyperlink ref="E31" r:id="rId55" xr:uid="{F2E5E1EC-DFA1-4DA3-A209-010E74727758}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>